<commit_message>
Planning PMS+Inauco Rev.1: ESD/F&G/PSS, FAT Maqueta cliente e integracion en sitio
- Nueva linea ESD·F&G·PSS: tablero marshalling HIMA (lead 25 sem desde JUL -> 23-DIC-26)
  + config/readecuacion PPSA (A DEFINIR, arranca AGO, FAT completo al iFAT)
- FAT Maqueta PMS recalcada como requisito del CLIENTE (22-25-SEP-26)
- Integracion PCS<->PMS: en fabrica (Bs.As.) + instancia EN SITIO durante el iFAT
- Actualizado Gantt (4 swimlanes), flujo, planilla y notas. Arranque Inauco 1-JUL
</commit_message>
<xml_diff>
--- a/Constructibilidad/Análisis generados/Planning_PMS_Inauco_CPF2.xlsx
+++ b/Constructibilidad/Análisis generados/Planning_PMS_Inauco_CPF2.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -687,12 +687,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PP-MQ</t>
+          <t>★MQ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>FAT Maqueta (prueba temprana, AESA)</t>
+          <t>★ FAT Maqueta PMS (prueba temprana — pedido CLIENTE)</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -704,10 +704,14 @@
       <c r="F9" t="n">
         <v>4</v>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>witness AESA</t>
+          <t>REQUISITO CLIENTE · witness AESA</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1440,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>INTEGRACIÓN Y CONVERGENCIA → RFSU</t>
+          <t>ESD · F&amp;G · PSS  (HIMA + PPSA)</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr"/>
@@ -1450,43 +1454,39 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Integración</t>
+          <t>ESD/F&amp;G/PSS</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>★INT</t>
+          <t>HIMA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>★ Integración PCS↔PMS — Pruebas ABB Bs.As.</t>
+          <t>Tablero marshalling HIMA (provee ESD/F&amp;G/PSS) — 25 sem</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46442</v>
+        <v>46204</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>46448</v>
+        <v>46379</v>
       </c>
       <c r="F34" t="n">
-        <v>7</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
-          <t>PUNTO EN COMÚN</t>
+          <t>lead 25 sem desde JUL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Integración</t>
+          <t>ESD/F&amp;G/PSS</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1496,49 +1496,45 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Inicio campo PCS — Sala INS (Sala 7)</t>
+          <t>Tablero marshalling HIMA listo</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46463</v>
+        <v>46379</v>
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>ancla campo IN</t>
+          <t>para FAT SIS / iFAT</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Integración</t>
+          <t>ESD/F&amp;G/PSS</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>★iFAT</t>
+          <t>PPSA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>★ iFAT — SE#3+SE#4+PMS+PCS+SIS</t>
+          <t>Config. y readecuación ESD/F&amp;G/PSS — PPSA</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46563</v>
+        <v>46235</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>46582</v>
+        <v>46562</v>
       </c>
       <c r="F36" t="n">
-        <v>20</v>
+        <v>328</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1547,35 +1543,31 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>PRUEBA INTEGRADA</t>
+          <t>A DEFINIR · arranca AGO · FAT incl.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Integración</t>
+          <t>ESD/F&amp;G/PSS</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PREC</t>
+          <t>◆</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Precomisionado (EL + IN)</t>
+          <t>FAT ESD/F&amp;G/PSS (PPSA) completo</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46632</v>
-      </c>
-      <c r="E37" s="3" t="n">
-        <v>46660</v>
-      </c>
-      <c r="F37" t="n">
-        <v>29</v>
-      </c>
+        <v>46562</v>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
           <t>SÍ</t>
@@ -1583,45 +1575,23 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>banco + campo + punta-punta</t>
+          <t>A DEFINIR · antes del iFAT</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Integración</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>COM</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Comisionado integrado (EL+PCS+PMS+SIS)</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="n">
-        <v>46653</v>
-      </c>
-      <c r="E38" s="3" t="n">
-        <v>46740</v>
-      </c>
-      <c r="F38" t="n">
-        <v>88</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>88 d</t>
-        </is>
-      </c>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>INTEGRACIÓN Y CONVERGENCIA → RFSU</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1631,25 +1601,201 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>★INT</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>★ Integración PCS↔PMS — Pruebas ABB Bs.As.</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>46442</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>46448</v>
+      </c>
+      <c r="F39" t="n">
+        <v>7</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>PUNTO EN COMÚN</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Integración</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Inicio campo PCS — Sala INS (Sala 7)</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>46463</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>ancla campo IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Integración</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>★iFAT</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>★ iFAT — SE#3+S#4+PMS+PCS+SIS (incl. PCS↔PMS en sitio)</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>46563</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>46582</v>
+      </c>
+      <c r="F41" t="n">
+        <v>20</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>integra PCS↔PMS en sitio + ESD/F&amp;G/PSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Integración</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>PREC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Precomisionado (EL + IN)</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>46632</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>46660</v>
+      </c>
+      <c r="F42" t="n">
+        <v>29</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>banco + campo + punta-punta</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Integración</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Comisionado integrado (EL+PCS+PMS+SIS)</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>46653</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>46740</v>
+      </c>
+      <c r="F43" t="n">
+        <v>88</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>88 d</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Integración</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>★RFSU</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>★★★ RFSU — READY FOR START UP</t>
         </is>
       </c>
-      <c r="D39" s="3" t="n">
+      <c r="D44" s="3" t="n">
         <v>46741</v>
       </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
         <is>
           <t>SÍ</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>objetivo</t>
         </is>

</xml_diff>